<commit_message>
Aggiornamento automatico bandi 2026-06-03
</commit_message>
<xml_diff>
--- a/bandi_campania.xlsx
+++ b/bandi_campania.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPVDGroXpPoAVZiqWR'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eij29DRSYSSA7Lr9b'}</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSSPSjnQvLzk1apDqu'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hoDET9bxFTez9A1CX'}</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSUctbQ3s7TgTnNRUa'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hrebpgF4WTkGFMPXB'}</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTCfEA2UJAHBw3shzz'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2it5hXyBVBYpLMb3gT'}</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTDHBXnLTPA89z5PHQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2itjeBiynxdHgfEMJU'}</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPVoVbgmeFjVwDz6jA'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ejRCFdx67TDSorerf'}</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPWHWo11Hgh2qn7L2g'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ekNjvGrvWsp9dXo4D'}</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQTj1GT89eQxCGidzf'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fVixYrdiBPJgo2S1G'}</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQUGkDHsS8oHvKQthe'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fWJgiZuUJowkSsFgZ'}</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQUwgAKQk24soHF9hB'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fWv9XBdNN3rZMuJ66'}</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQVebXDnofQRT1e3iQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fXtvzy8CntdrfGiWF'}</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQWcPGdg6RKGqrVNbe'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fYTQqE3RKDujd6g7Z'}</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQXEbVs4aovhzKv4Lv'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fZ1enqbkFGpg77QWj'}</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQXmqUNDqczR6bSnaD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fZc7oAUzNvusm3LXo'}</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQYHbRh8ATRcoQqysu'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2faC6B8iehFjC1VHH4'}</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQYqq6PTjakbFMHZSh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fbA8wfs23AqmBddDn'}</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQZQozgEgrGRNyDDL3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fc9uwbMLU2FGDe1xx'}</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQa8y1sK4HwLdXEHuV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fck8hBzDtYKjgsxL6'}</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQagTiLXE2tNonhu3L'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fdL7JfXhVmfQMBpAU'}</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSU5PdW7MsL929uQqF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hq8pNXstsuJ41WAV9'}</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPd1aSSuBKZ8V18vm1'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eto12GGB5Gd5aGzJK'}</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPHNdWd9srBv1j74Rm'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eZpjzaNSvqFD1Z8Bo'}</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT7VReAJAQx8EBxJUp'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2imXZQMH2ERrdq1c3k'}</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSbFzPkVYDNEtkHrQz'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hz5awzv5vwpYW6VZe'}</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRkTbvQxtqCtk5kNgy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hEvHDGA9xKRNCeR3Y'}</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS423HZpEp4D7fcMZF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hZzVWihupHM2t8byz'}</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSFmECpv1Z6rspKiUw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2heBWKvdE6nqzLYwcT'}</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPJbo5zdQY46x4Lnyg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ec1CiYxVTajFZPAnw'}</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPKRQtqWN2c7TmYRqj'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eccv87XNHjmGjDjMs'}</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPKz92E78tfsg6qdeq'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2edDP32ZLHtURnuV2z'}</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPLrjK9hrEwvTJRQw5'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eds5DsfyPNDXyeCzT'}</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPNRjnSXEj8r1g8P1s'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eeVmn3sMC9cCPKc9G'}</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPNyj7cMSBF3Uqycco'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ef7Efcm17LL6P1W6K'}</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPPcvTcTfT96ccPsxE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2efmRh42J2NxxE8bkh'}</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPSK9PPyNNxXgcycws'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2egL9x2fiZg92HoeAo'}</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPSpuPqmuKvBVty5hK'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2egxMhYG73wKq6Fn2S'}</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPTWaRiFx8nNq3iXZV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ehYLUj55Wmv8zdbYV'}</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPU8XmxCtastMFsKxR'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ei7ox4UPaWBd1ZB8T'}</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPWwxC5MvzFDjRfzwC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ekyTKvLWq5oY5wKxk'}</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSJNjn84HvdRckPwMg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hgeqS2R35Ra5gx3xd'}</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSJxxnHvoabeEA2B4N'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hhNVhCa4ihWBLUG6t'}</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSKUTzqQvHLbw7efre'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hhuVjBCCf8Vao2Gpv'}</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPmr9Dqw4o5HrPvVpr'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2euRTGyaMyqt36wG38'}</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPY4g2AMno2ybRcUzC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eobxxyKrr72HE8fMe'}</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRSoxrMLyfc5W25Uyc'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2grvwnMTx1576xSPvb'}</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTBY1FkwzLP2YGgGHC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2irj6YgR5gGRZoKb2a'}</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTC5zmqU9vW96hUXLX'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2isK4rJsgpv8X8noQc'}</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTKAteMoXdSeHUdnmD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2izh5Kbp3JWTbWhfit'}</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTMKd1NnZSBH1Ht2gB'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j4fwVeWUy4HfhUors'}</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTQkVjpeQjNvk2QG6r'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j8sSrpuQRSbU5R11c'}</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTRGkfsNwBX2rSoViV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j9Sg4Wvxf9yiN2e28'}</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPHyqc72VJ93wZibfE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ebRjSEA21qiPpy6f2'}</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSFBFpMn64C2eCfpbe'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hdbnKEjjB5p3x3v6a'}</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRTea8bX1WitFc7JWQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gsbNvvoCvJhtPvLia'}</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRUBKC2fT46eAYNY9J'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gtK2wsV1kSso2Zbue'}</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTLo7j9sLFhBbvQBqT'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j2ZgjyvG9exM9RxWa'}</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTMscWHNNB2x7J8g91'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j5EftZpKWFLyU24Uk'}</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTNb29TWvAKMcsfwu8'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j6MtHn2vnr661CU4h'}</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTP6HLvsurQA2H5J1y'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j74YzLhRD6k95d4GR'}</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTPeGpJ9AgKFhvVjJb'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j7dHT1q3a8a514FA3'}</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTQBX33M5p2fUKqugV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j8EFgYvnvee17fR6w'}</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTRpzGLnFm2EV8kmhN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2jA1ucXuPuBgBPTmuc'}</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPbq8wbWvGT9cDShhw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2erUrQpWvXr46sR27i'}</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQbEwax484moyX9Vhw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fdwZnp7oUKkurPXz2'}</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQbnSDzkwCcVfUCQJN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fyVK1kU1J6XvbohfV'}</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQcNfFZuKKUQKa9mgM'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fzruVQ8tfjm8rrx5X'}</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQczNGj5C8uCVsvNm9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g1WrNHoJTX3vcpthe'}</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQdYbvYTzJrm7y9Lpp'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g2FkMqPjFJGT91MtP'}</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQeAZTUZjPXKZJdZqC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g32soZCjeuq23tfzL'}</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQehoYXAgSZ4e3UajV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g3brtg79CGN8xSwDQ'}</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQfWvGd1n7JmbB2KkP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g4BauZgWtH7zfqthq'}</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3906,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT8c974sMPsdXdMmgn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ioWcgBgTSHXC5SaP8'}</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTKisin2DHk2BznebC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j1JXpFGRfjVhbHrXQ'}</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTLFsYH8QPjSpDNwnd'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2j1rmZUdmp5U8T4CtX'}</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTGpkQTh1BKrdGcxht'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ixGUJRTuRtjmgiCBm'}</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRJwh495mMmxdx8eMk'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gj9dN3BcgdbHfjhdZ'}</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRKWg7c72mWBJMH6Ex'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gjkqVdLUkiiwfyPXx'}</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPrd8QkTsXaSsDc1qq'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ezpu1puqfjKNJYzRg'}</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPscAPfmr1NUcQBkxh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f2NR5z4EiXSwsbest'}</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPtn7La3i9QnRWi5U2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f336iBXPu4WvFPg3n'}</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPuLbNsRR1fN1xioE4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f3bLXha6xrsF94UQF'}</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPurMZBEfb7Pb8fvoM'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f4A4yFmDqFo2t7G4P'}</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPvSaNjW6BAA1Fn4fg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f4nGhTw8dF1JPVQhU'}</t>
         </is>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPvypCYMVRcSsdWhdh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f5aQ7Ln8jNJ747S6d'}</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPwa3MBFfUFo1i1UBy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f7NYRoiEXsXubvi7y'}</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPxX68tEUDKjDckbj5'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f7y1xnUfDdMrThede'}</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPy5aM1Tj8neBdtNHs'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f8gg8DYisnWCXHMTr'}</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPycpNMJHyowiEqXKN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f9Lch8mTj8Z4M6PZn'}</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQg9NSrEhGho6CWrJF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g4kov3Hopd446omAm'}</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQgj6RtCiLCfMBwHCm'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g5PWhGvS3gyVeu1Ct'}</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRLH4FYedxvjs24oYW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gkNnzfUmXXU6zYBam'}</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRMLJqnnei9798hbEH'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gkyGGE7UhfzQDYJuH'}</t>
         </is>
       </c>
     </row>
@@ -4893,7 +4893,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRN1VNJdLXabQJhqDW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gmzmyqdaijYGVHjjf'}</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRNW1JKJ2U4iiF4FZZ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gnaFzgLdYezaz5SQK'}</t>
         </is>
       </c>
     </row>
@@ -4987,7 +4987,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRP3VujR4MPbg7eojL'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2go9jSQe3dsEWnjahN'}</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRPqdHy4cYmNwUd7A5'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gojCujzmNzU5iaNgY'}</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRQcWVVU5DT8bDTg3E'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gpJgf1dwEDSLyTX7j'}</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRRCUnV3EVvaCe7B3p'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gpx8XJtGBwiyiQLei'}</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRmEVE3krAuqWY5Ex9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hFYjNBTa4Xff9ASQn'}</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSEZnyJAEVUZLybz8T'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hd2ohPuhujHcWEpEs'}</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSL6RjeDmCcncVmNvP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hiUyTeBwS6AVU8pFt'}</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSLh96kxPQgfocjDU3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hj4SjPmXMYM7Bn7a2'}</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSMH7gkk6emo9JQ97U'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hjgtxQ4Ev3YUNgLs5'}</t>
         </is>
       </c>
     </row>
@@ -5410,7 +5410,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSMs5nDW7Yoyvz8oCg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hkK7C41F7qkLwLJAY'}</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSNVYPeiyU8uKeTm1J'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hkua2Anryz3t4UHcF'}</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSQ1Kn4aJMivtVJRkh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hmUoUcTGtQvh83tfL'}</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSQfWWtxAj5xL9ge1r'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hn42eQKPzq8QhJGwA'}</t>
         </is>
       </c>
     </row>
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSRMgdiM7QW8n13mZy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hndWXCJQrKQXuAceh'}</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT99dxDVzTmcTxNRnP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ip9597bqueHFpSit4'}</t>
         </is>
       </c>
     </row>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT9feJXnnrVpfn5jWE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ipvhZus6J8pCCbykf'}</t>
         </is>
       </c>
     </row>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTDvNiZwze1h5uMLKF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iuLcNMebcmnNho4Jc'}</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5786,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTEVrNNpxchaqrgJHt'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iuy4TwYzPBZ6BqhB8'}</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTF17n764L8yW5XsZw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ivXnz1osQJR8g93Td'}</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTFXcTx91Reo2j3WPW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iw729bzMQHFXjuQ12'}</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSHZNo8MQF2gVyAc5h'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hg6MHHbpUJqmWtRy4'}</t>
         </is>
       </c>
     </row>
@@ -5974,7 +5974,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSobePgEmY6MF5Tjdn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iFDfWjJCptcyAXujY'}</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSpQGeoSMPPz5P8Xfc'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iFpdCgZd62tfyeUNZ'}</t>
         </is>
       </c>
     </row>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSpwGDA7RiaAUcbWjy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iGQ78Lh7D97yYM3YA'}</t>
         </is>
       </c>
     </row>
@@ -6115,7 +6115,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSqVzqydsS2fwY1exP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iH1p3fnShMSA1XrBF'}</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSr2zWMPD2MHdkQsAS'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iHcHMUPed6kJtDwRN'}</t>
         </is>
       </c>
     </row>
@@ -6209,7 +6209,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSrmPoBthHcDLXSBPL'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iJDVMVGywPLGifDur'}</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSsHQ5jenKowHtXxSS'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iJoxu8KBDMCcFXscr'}</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSsouTEz4smyeunEFQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iKSumFajXJFKVaFz3'}</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzStQsJ215aKwpo9rUh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iL4NV6ewLujGmNcxn'}</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSu82uhYCjGpycZQ6g'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iLdqtq2eEfAHiBbMM'}</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSudnTYRfSCmwpKJar'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iMFZEJXGUu9jNVpVQ'}</t>
         </is>
       </c>
     </row>
@@ -6491,7 +6491,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSvBn1wD4gHE9c73ZU'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iP6gDzkhnoigkUPbk'}</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSw5rTDFJTWE3D7wdf'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iQ1W5VY2qpTzRCVvH'}</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPcPNaZZDTAvHekE7z'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2esB2AstHE5wqAMz6V'}</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPzAoiy7zQpGbH4PXv'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2f9wLMKMNR9gAPgZJL'}</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPzkHB9SatotD2orTy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fAgEAnHpsjhmmCt4r'}</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ1PyQEzKZo5mNtU86'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fBJBxR73MGQ4wpzQc'}</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ2UTvEBBJB4Wq3XEa'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fBsfZGkSArh2qykBz'}</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ32hrYRS4gAuxatxv'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fCVNeB1mwSRqtaTvG'}</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ3cRdwWFt9kfnpqZB'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fDHzP9E23AotEccuy'}</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ4AAjjuUjixajRzSe'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fDrixGhfTp3Az4sHU'}</t>
         </is>
       </c>
     </row>
@@ -6961,7 +6961,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ4hAVt5ur7xEg4phy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fEWfarY2Uu3HvfFDo'}</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ5FtqL1SNg3ChfPtM'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fFSDxe3ycz1uzhATo'}</t>
         </is>
       </c>
     </row>
@@ -7055,7 +7055,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ6Fg2KhFnAUF5aNiy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fG4Rx4Qr5gtSPsGNa'}</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ8Nv6JWt1rLir4Y3y'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fGdfS1pnV1mnG5ga9'}</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ95arkLhuQ931wmiV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fHTGThWgwruP5FDpb'}</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQ9cae4SunrgqKAWa3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fJAC1DfyBDQbbfcU2'}</t>
         </is>
       </c>
     </row>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQAE3LeUhbXxNxsMr8'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fJkA4abAboweboQrW'}</t>
         </is>
       </c>
     </row>
@@ -7290,7 +7290,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQAkYKuHcpTMmdKEK2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fKL8Zw5KNFJ4dEexF'}</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7337,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQBJXxdyFRYTZ6ffv4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fKwLuM5WCAEidSUPb'}</t>
         </is>
       </c>
     </row>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQBp3CEmDdmhHPR7vj'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fLXpC6V6NYUcYyn8z'}</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQCQWmLjFFEHJhz7Vu'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fM92XZTuqZ8SqQtRx'}</t>
         </is>
       </c>
     </row>
@@ -7478,7 +7478,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQCzEZLSY7LmFnXXK3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fMzNhDwhkVZrRToWB'}</t>
         </is>
       </c>
     </row>
@@ -7525,7 +7525,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQDi9H1b6wjwVWdyXj'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fNbqAfyc6B1P7uR9s'}</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRimAQge6nTjCpp3mb'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hELYotjYBJTBxnye5'}</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7619,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPXYv1FAor5iE32JEF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2emwVzFs4jnzjfuBjq'}</t>
         </is>
       </c>
     </row>
@@ -7666,7 +7666,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSbnz6i3suzyDZDzvn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i11tRX56oVz1eVw5u'}</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7713,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzScMy4JbsU37E8EQuD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i4E879tFLz1Bg9GQf'}</t>
         </is>
       </c>
     </row>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSctidEGyGzxCeNgqs'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i5ynnGZ2gdXQYUFuT'}</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSdRxeJcWMhYswXg15'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i6ghey8Q3eACJWP1j'}</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSeyUjda5CQHhNuBnR'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i7QNLYNTcSJtUM98U'}</t>
         </is>
       </c>
     </row>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSiGg496jTXXXJvqQn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i9mVig8dPi5Gxsppg'}</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7948,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSjY5F62nhsj4PQ1iN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iANi2emirQ4FoM1kC'}</t>
         </is>
       </c>
     </row>
@@ -7995,7 +7995,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSk551kR1rK24vJVm7'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iAyvRaatzoopX9aWV'}</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSkcohvgXTHtj7urq1'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iBZPqD8rZv4wFdBa5'}</t>
         </is>
       </c>
     </row>
@@ -8089,7 +8089,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSmD2a2mQBjqNgxpVY'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iC8NzutvnkKusG3SA'}</t>
         </is>
       </c>
     </row>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSmqV7owy4J6GR1vcr'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iCibiZgss82bQi4kX'}</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSnPxtQuifALxLinxD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iDbgNUcP8CLZtBvWm'}</t>
         </is>
       </c>
     </row>
@@ -8230,7 +8230,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSnuE67bheTNngiJ1W'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iES37ENvSJRoaj6RN'}</t>
         </is>
       </c>
     </row>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSxSTX5wrTxgSW5Haw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iR9i9jnSkGPbirWkW'}</t>
         </is>
       </c>
     </row>
@@ -8324,7 +8324,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSyCMEynEXeVu3GWgg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iRnQZDh9dDFM6gGX3'}</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSynZuZYHmM4dB29eW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2idVrfukumVPvk2dvm'}</t>
         </is>
       </c>
     </row>
@@ -8418,7 +8418,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSzQ2yWz2QMa8yV8DF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ieRvEANaAvCjbTSu8'}</t>
         </is>
       </c>
     </row>
@@ -8465,7 +8465,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT1G8DKseGaN9sW2tJ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iezejF98YimM7Yxhh'}</t>
         </is>
       </c>
     </row>
@@ -8512,7 +8512,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT2kAifZbf1f2ceVGW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ifbcc4CzZt2GBR1fY'}</t>
         </is>
       </c>
     </row>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT3GvPATCEDRmdwbHE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2igB6TuZtrVCEFKfkg'}</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8606,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT3nvNbMEYYAq3Q8Jy'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2igiqPnPx6ejf8XR7r'}</t>
         </is>
       </c>
     </row>
@@ -8653,7 +8653,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT4Vb8nLSJR3PAsrnP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ihHKNmgPNWsnsQ25E'}</t>
         </is>
       </c>
     </row>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT5Mvy8HogJiQpKQK3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ihsY5f97QikzXjBkK'}</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8747,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT5uRgEND6b26TAYzf'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iiahYAbrHY1yAw3p5'}</t>
         </is>
       </c>
     </row>
@@ -8794,7 +8794,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT6TuiVVFKUb9aNMHd'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ijQ4fy7zs3QsMc37H'}</t>
         </is>
       </c>
     </row>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT6yujuYwY7oVytrWr'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ijzHYkwHF1B2Apveo'}</t>
         </is>
       </c>
     </row>
@@ -8888,7 +8888,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTGFGkiNyoyA7MP2n4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iwfkqFP9t3rfTUfeb'}</t>
         </is>
       </c>
     </row>
@@ -8935,7 +8935,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPpF1H4avGDS2es1MP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2exDPNv9gAkvWbBRTn'}</t>
         </is>
       </c>
     </row>
@@ -8982,7 +8982,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPpm1mM2MnHaw92CrN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2exqLsQV9BvKV7bBFJ'}</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9029,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPqGX7BTbvYQ1miy1Y'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eySJXQ6PhvadzU4Mi'}</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPquUF9pBLLfm8uyLb'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ez4kiFSfBHNwQ9hk2'}</t>
         </is>
       </c>
     </row>
@@ -9123,7 +9123,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQhrZeU75yMNf3q3Pe'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g6ff2rkz6PsvqBuPL'}</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQiX14WT3iUCy7mviJ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g7E9MZ8A6M428nAsF'}</t>
         </is>
       </c>
     </row>
@@ -9217,7 +9217,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQjJdMc76kQMmcQDx3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g7oNNmMXLrwXhJKQg'}</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQjp8jxmrtWHeJs3b2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g8PLs5SmXw9PJDSxi'}</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQkN8BoVep4ppGH2sz'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g93XuDrWq4YRp4owU'}</t>
         </is>
       </c>
     </row>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQku8556csiNTGQW9t'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g9fF2W3QeNh6JPdeF'}</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQmS7eYSFc77HVfWfd'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gAmiSJLZPtUsYP8Vo'}</t>
         </is>
       </c>
     </row>
@@ -9452,7 +9452,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQn2LPhLWVgtnrWkFA'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gBNg9YuxH2NT9s1P2'}</t>
         </is>
       </c>
     </row>
@@ -9499,7 +9499,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQnZ5mYkNMAgkcmqga'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gCLUYPzT7Cmaw7BiV'}</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQo84eiNXDbhnCzDyw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gDDoZZGCCc694K8uT'}</t>
         </is>
       </c>
     </row>
@@ -9593,7 +9593,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQogYpUKT6snfUJbxx'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gDtzA1LxzpJSVcAAs'}</t>
         </is>
       </c>
     </row>
@@ -9640,7 +9640,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQpbNGv5o6wn4DNoUc'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gEuWQpEWJyTKVGfVS'}</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQqB6Fma5qtece6RsE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gFXDJnNHtnMoGnoyj'}</t>
         </is>
       </c>
     </row>
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQqmopjbtYmRGcyrq9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gGdBrHaF6sNSBKuF2'}</t>
         </is>
       </c>
     </row>
@@ -9781,7 +9781,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQrKoGQZu37tJwMN23'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gHZVdV41yYrDzC8xa'}</t>
         </is>
       </c>
     </row>
@@ -9828,7 +9828,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQsZxWxyMQkYt17Q3p'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gJ9UJZcseos3dJWPD'}</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9875,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQtDQKBwBYnrydbxr8'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gJhhxsqyFrKYFtm2t'}</t>
         </is>
       </c>
     </row>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQuRqFq5mqDW14k5j9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gKFwik1Qhu9pNz7ms'}</t>
         </is>
       </c>
     </row>
@@ -9969,7 +9969,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQvDTXDju2yMvawZEA'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gKteDwLiyiwo3VzHT'}</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQvkhXjTYDP1Ak2672'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gLcoKGQhMQWvPtC6J'}</t>
         </is>
       </c>
     </row>
@@ -10063,7 +10063,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQwHCwovFpbSm255Mi'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gMCXKnhyLMs51NygQ'}</t>
         </is>
       </c>
     </row>
@@ -10110,7 +10110,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQwqw8FxZYCc2JSNNw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gMnVqEK6yAk9QHUCF'}</t>
         </is>
       </c>
     </row>
@@ -10157,7 +10157,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQxQuwdeVCL9YEbcER'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gNZt2GKQLwtk21N6Z'}</t>
         </is>
       </c>
     </row>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQxyQHwWmjKFdvmt9Y'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gPYATRES79Rk1HBVG'}</t>
         </is>
       </c>
     </row>
@@ -10251,7 +10251,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQyW9WGgGJC7v6S4VZ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gS2jTQDunHhfmTzGE'}</t>
         </is>
       </c>
     </row>
@@ -10298,7 +10298,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQz3PtDf7LFG4CVT1y'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gSxYcGcPdquC89MrD'}</t>
         </is>
       </c>
     </row>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRUjoUiEYM6EQv787A'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h6RJkRVci1PgNwEFC'}</t>
         </is>
       </c>
     </row>
@@ -10392,7 +10392,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRVHJ3MSvxMuSqEAk1'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h7azvLiEcAjLnJvyT'}</t>
         </is>
       </c>
     </row>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRVr2huQk1kQGRvAX9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h88VXpWRqieRRWB6B'}</t>
         </is>
       </c>
     </row>
@@ -10486,7 +10486,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRWM38E3xKHHi8Rfwo'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h8mC8zBPTFCLJWGUX'}</t>
         </is>
       </c>
     </row>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRWs3bK9yvZXtjwsKB'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h9LRWBXgR5iFGK64v'}</t>
         </is>
       </c>
     </row>
@@ -10580,7 +10580,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRXPoEyKYFZq2sZxMo'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2h9vtT7SZrz6LpebCu'}</t>
         </is>
       </c>
     </row>
@@ -10627,7 +10627,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRXyWzq86jKR2yKdPx'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hAcZeSWkWZxUnCMzc'}</t>
         </is>
       </c>
     </row>
@@ -10674,7 +10674,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRZEg5wkvkVCgtfT3V'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hBBoHPvncHuaaqLC8'}</t>
         </is>
       </c>
     </row>
@@ -10721,7 +10721,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRbMv2gYR9YqqwBtvc'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hBoFy1pHwMmQsLRQS'}</t>
         </is>
       </c>
     </row>
@@ -10768,7 +10768,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRcdoyYWpPtjEnabep'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hCRD5VXPSA9U9NXHu'}</t>
         </is>
       </c>
     </row>
@@ -10815,7 +10815,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRdH1NWkigybwkjyvH'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hD4fB5aNKPpfzmMH6'}</t>
         </is>
       </c>
     </row>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRgnMLsG8qLhfCKsCD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hDkpxdBunKkZZ6AWh'}</t>
         </is>
       </c>
     </row>
@@ -10909,7 +10909,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRmjkfJhb8W4nMjTs5'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hG9waJZ1YnbXcPMU6'}</t>
         </is>
       </c>
     </row>
@@ -10956,7 +10956,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzT83ugpLjuL3yxrvLg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2insfqiVK2zsEZbNRE'}</t>
         </is>
       </c>
     </row>
@@ -11003,7 +11003,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQze7LFFU5qEW7mKkp'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gTiSCPQoxTVg14TkZ'}</t>
         </is>
       </c>
     </row>
@@ -11050,7 +11050,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRHuw7sa7kSFCueZcz'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ghqW1vxkAJixGoueG'}</t>
         </is>
       </c>
     </row>
@@ -11097,7 +11097,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRJRwQ3Efy4hgQzY1i'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2giYfdQ1s7CtxQ6qFH'}</t>
         </is>
       </c>
     </row>
@@ -11144,7 +11144,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTJXweNMZTNXThQUm2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iz8axEhyR2wefbibe'}</t>
         </is>
       </c>
     </row>
@@ -11191,7 +11191,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRnRgAPioPLnSFXfuj'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hGmtuQeXp28wwUcs9'}</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRnwBS6vZmq9ZfY76U'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hHNcXPgDin4km7Egb'}</t>
         </is>
       </c>
     </row>
@@ -11285,7 +11285,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRocrrgbNxJPBHsqwQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hJ1ZaKZrSc5RjD1i6'}</t>
         </is>
       </c>
     </row>
@@ -11332,7 +11332,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRpTxSyxu6yBaQ8N7W'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hJbHdhrMugTSMMGe8'}</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRq6ALpzmdmHE1M7ja'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hKNfeJiKnyLkpJhai'}</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11426,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRqwkmdFpbcoZfr2pL'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hLWsnhXW5BfGJKxAw'}</t>
         </is>
       </c>
     </row>
@@ -11473,7 +11473,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRrTGeSkeLg4w4aMTD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hMKzLwF3TtBMwULX7'}</t>
         </is>
       </c>
     </row>
@@ -11520,7 +11520,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRs1W22xYD26DHrh67'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hMxh2i5N1oF7RjKUL'}</t>
         </is>
       </c>
     </row>
@@ -11567,7 +11567,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRsZVfFWcRHZ7Vj6SG'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hNb9WN6g9HTfJqZ77'}</t>
         </is>
       </c>
     </row>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRt5zebcn7qNsz9BPw'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hP9PFKEvsbAqrKcAn'}</t>
         </is>
       </c>
     </row>
@@ -11661,7 +11661,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRtcViquo7KQv65R8d'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hPicWowjnf4xemmWX'}</t>
         </is>
       </c>
     </row>
@@ -11708,7 +11708,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRuy6tBzKe4K4qwCRp'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hQJ629qwnnS9J2KAB'}</t>
         </is>
       </c>
     </row>
@@ -11755,7 +11755,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRvYai22xSKeDUz7tm'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hQsZWJa8xNYS9PoXG'}</t>
         </is>
       </c>
     </row>
@@ -11802,7 +11802,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRwAnUZJMmXWDoMbF4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hRS3WHXnSCpXV3G2m'}</t>
         </is>
       </c>
     </row>
@@ -11849,7 +11849,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRwi2UuV1dkeMTUrBu'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hRzn3QLdkidqyzSRQ'}</t>
         </is>
       </c>
     </row>
@@ -11896,7 +11896,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRxc6tk6aqVd2P91bo'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hSbVxWv3pnRScZmQe'}</t>
         </is>
       </c>
     </row>
@@ -11943,7 +11943,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRy7cTh4pKgMUHYpvQ'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hTECb7E4hQ1MJKp5E'}</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRyecFYqwP5cqRtq9v'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hTrenJhDEnd6jr61P'}</t>
         </is>
       </c>
     </row>
@@ -12037,7 +12037,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRzELWrCb1cvR8UoG4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hUTcN8s3Rm9wYst6U'}</t>
         </is>
       </c>
     </row>
@@ -12084,7 +12084,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRzjbSLvc2L6y3W51n'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hVHiormB8F85z6vN9'}</t>
         </is>
       </c>
     </row>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS1GbURU2hk8SbiUNi'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hWA4MFFWzAAxR18W8'}</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12178,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS1r4kADe5ztKV3xi2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hX29k7pDC2GB5QGAs'}</t>
         </is>
       </c>
     </row>
@@ -12225,7 +12225,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS2PZSGtRWJNf8JP65'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hXfLz29wW8qr4x2mz'}</t>
         </is>
       </c>
     </row>
@@ -12272,7 +12272,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS2voYo3kWC3MnqPfn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hYYgRXjDhtHXiJdTf'}</t>
         </is>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS3UYYt6xzzF7La5Wz'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hZ7uUttyP4BVmMKjB'}</t>
         </is>
       </c>
     </row>
@@ -12366,7 +12366,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSGUe6iUsH3HF5i4Lo'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2heoU9DCihX82M1UUH'}</t>
         </is>
       </c>
     </row>
@@ -12413,7 +12413,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSH38AKvdLFybTVgAx'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hfXNgxg8Rsa2XZnhC'}</t>
         </is>
       </c>
     </row>
@@ -12460,7 +12460,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTAVVr6DYXgEE22tEb'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iqXundcAg7GQoyKY6'}</t>
         </is>
       </c>
     </row>
@@ -12507,7 +12507,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTB1FxZv1KmZB3mbsP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ir791i552MzLc1RcW'}</t>
         </is>
       </c>
     </row>
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzS4ZXnvY8dtQBSMwxr'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hbHdbdaufkTYtSeeX'}</t>
         </is>
       </c>
     </row>
@@ -12601,7 +12601,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSVAP1rWooYdKJNgjR'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hsdPbCxXicxtwY1uq'}</t>
         </is>
       </c>
     </row>
@@ -12648,7 +12648,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSVgt2M2tuZJXcSVRa'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2htKZdiAMhYZKLWcZu'}</t>
         </is>
       </c>
     </row>
@@ -12695,7 +12695,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSWDNtRb3sCqn6wTe7'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2htvmeVVLwLuqkwfaM'}</t>
         </is>
       </c>
     </row>
@@ -12742,7 +12742,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSWorFvF55q7cUPs57'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hus5XJaVGkZxZiuNE'}</t>
         </is>
       </c>
     </row>
@@ -12789,7 +12789,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSXx4W48utquKGpiG2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hvvagjUX5JBKKgmwE'}</t>
         </is>
       </c>
     </row>
@@ -12836,7 +12836,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSYoACts1mqcXzuzwa'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hwnRFjwTkFK7VVssF'}</t>
         </is>
       </c>
     </row>
@@ -12883,7 +12883,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSZJv3e56169d6XJwE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hxM9vDcbQ8hvo7j4c'}</t>
         </is>
       </c>
     </row>
@@ -12930,7 +12930,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSZudPZABaQ7rcu8VL'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hxueApAARd4XrGYnq'}</t>
         </is>
       </c>
     </row>
@@ -12977,7 +12977,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSajF4jnGSz297F2Ga'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hyVrfcxZt2tP8ApSA'}</t>
         </is>
       </c>
     </row>
@@ -13024,7 +13024,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSwi432LK9KwwJsPiN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iQayPuHKuVGWVbjRN'}</t>
         </is>
       </c>
     </row>
@@ -13071,7 +13071,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPnMQCDg4twgzsMBEs'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ev1fzPAmTcgQQtoxM'}</t>
         </is>
       </c>
     </row>
@@ -13118,7 +13118,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPnu9Ra1H48NjXHjDh'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2evd92fsY4At4d9VtB'}</t>
         </is>
       </c>
     </row>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPogmtrBrnSaXRFWM2'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eweA7xPq9GLg9ayY2'}</t>
         </is>
       </c>
     </row>
@@ -13212,7 +13212,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQhKoxtRsEfbwktt4f'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2g61iZowwY5CgVoQXa'}</t>
         </is>
       </c>
     </row>
@@ -13259,7 +13259,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSSvC6KiRmkUT9y3wA'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hovPqKr7pmbrBdVdM'}</t>
         </is>
       </c>
     </row>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSTVfnYAysawFHQ61D'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2hpYbiccSYVEW6nNaG'}</t>
         </is>
       </c>
     </row>
@@ -13353,7 +13353,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR1MH8vp3qLorvXe2m'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gUSqrad7DR1PeXNKA'}</t>
         </is>
       </c>
     </row>
@@ -13400,7 +13400,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR4Bw3zkbtdsqmEgvC'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gUzLYx764A1juNQr6'}</t>
         </is>
       </c>
     </row>
@@ -13447,7 +13447,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR4mekHm81v2Emqdxo'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gVcYAu86Ca2wWzZUk'}</t>
         </is>
       </c>
     </row>
@@ -13494,7 +13494,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR5KeTJU8HBqtZevB9'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gWHE4zbqh1Hf3pcBb'}</t>
         </is>
       </c>
     </row>
@@ -13541,7 +13541,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR5rtKtyQLpB1kXFEx'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gX6LpGLBdDgAVs59r'}</t>
         </is>
       </c>
     </row>
@@ -13588,7 +13588,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR6TrGJMNHUXVaTivE'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gXtxd3RAfR6eVYNsw'}</t>
         </is>
       </c>
     </row>
@@ -13635,7 +13635,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR7SeAECM8R4FtBNdV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gYUBirPzKLdrTXVjX'}</t>
         </is>
       </c>
     </row>
@@ -13682,7 +13682,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR8Rg55F6BTdFDrQzt'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gZGZEExPDGd3GncWw'}</t>
         </is>
       </c>
     </row>
@@ -13729,7 +13729,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR92dx4VicM6kqrrN1'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gZrXw1VpfCXf9UdTT'}</t>
         </is>
       </c>
     </row>
@@ -13776,7 +13776,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzR9e6dyT8Mg6RfxhnN'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gaUz3P8pHdV2MFbXD'}</t>
         </is>
       </c>
     </row>
@@ -13823,7 +13823,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRBftKnZcoytAkpihY'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gb5hPrro7Y8cWQZ1X'}</t>
         </is>
       </c>
     </row>
@@ -13870,7 +13870,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRCEs6oavTTtENV4VF'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gbfv9LGVe2Rs2B8qn'}</t>
         </is>
       </c>
     </row>
@@ -13917,7 +13917,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRCrpgBRz4dWp7s6dH'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gcGt7e6T8ipG7LJgC'}</t>
         </is>
       </c>
     </row>
@@ -13964,7 +13964,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRDSJViR2y8JAEaWCn'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gcs6r4wJZpa4EBcev'}</t>
         </is>
       </c>
     </row>
@@ -14011,7 +14011,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRDwK15SJD9sEZY2o7'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gdUoxpsLtHHdfsvwh'}</t>
         </is>
       </c>
     </row>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzREV44NWNDAAzatXvv'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ge3o6metqcbzJDSS6'}</t>
         </is>
       </c>
     </row>
@@ -14105,7 +14105,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRF2YiwiPbVMJXbqnx'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gebXpc2U63412uyqu'}</t>
         </is>
       </c>
     </row>
@@ -14152,7 +14152,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRFaHedNU7d1MWraHH'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gfNuvyygbq7VEJ7FG'}</t>
         </is>
       </c>
     </row>
@@ -14199,7 +14199,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRG9Gbqu7qY5gvVXHV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gg3M8PwMMuAxfmR4e'}</t>
         </is>
       </c>
     </row>
@@ -14246,7 +14246,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRGfGmPdnmPju37LAR'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ggcLHvKCHxg56sgiM'}</t>
         </is>
       </c>
     </row>
@@ -14293,7 +14293,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRHC29a4fDEEb48deA'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ghF2x1mTn5Ws5rrVK'}</t>
         </is>
       </c>
     </row>
@@ -14340,7 +14340,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTHUwPG1B81GGUq16M'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2ixx9eTYX2Sjgcs59U'}</t>
         </is>
       </c>
     </row>
@@ -14387,7 +14387,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTJ1SRsjUGJdSxSPta'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2iyYceX347PqThtxZ1'}</t>
         </is>
       </c>
     </row>
@@ -14434,7 +14434,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRRjEELuCktk8qN2RD'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2gqdonoSHubquaMgF1'}</t>
         </is>
       </c>
     </row>
@@ -14481,7 +14481,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzRSFyrSXC3hx1Sbq5d'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2grNDC7rw8sgRq6hTH'}</t>
         </is>
       </c>
     </row>
@@ -14528,7 +14528,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPbGex7F9dzqHTQ7sq'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2equ8DbPBqBrcpzG2n'}</t>
         </is>
       </c>
     </row>
@@ -14575,7 +14575,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQEJcW6x3yb3Jq8mMc'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fPG1yjZwfh7vDpFEA'}</t>
         </is>
       </c>
     </row>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQEqN2wXBBDRjmYUVV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fPtUQzh2Jqt6qpprt'}</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14669,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQPrbBji2ToZBWS4a3'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fQZQV5sGYwoAi3hkD'}</t>
         </is>
       </c>
     </row>
@@ -14716,7 +14716,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQQN6N5R8Dsk8fdVhW'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fRzUVgYgofp3nV1uT'}</t>
         </is>
       </c>
     </row>
@@ -14763,7 +14763,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQQz42nSjrqsEik6qX'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fSaCcB3UNQjixQovY'}</t>
         </is>
       </c>
     </row>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQRWYwsvGXMFvbYm6n'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fTEdxq3zcaN5iGLEz'}</t>
         </is>
       </c>
     </row>
@@ -14857,7 +14857,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQS3oA9puXgRbZA7Bs'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fTvZVE8pujXTwY9wN'}</t>
         </is>
       </c>
     </row>
@@ -14904,7 +14904,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQSbYEiBBX72piYGUV'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fUWY9jTw7Zuc3Yv7D'}</t>
         </is>
       </c>
     </row>
@@ -14951,7 +14951,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzQT92mYW8iZ8FPzCps'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2fV5m933v6ZL7u4xqh'}</t>
         </is>
       </c>
     </row>
@@ -14998,7 +14998,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPaARYoEkEWs3rwjGP'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2eqKu9c5KwQWNxKTih'}</t>
         </is>
       </c>
     </row>
@@ -15045,7 +15045,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTSzw23LsFjLYz8DpY'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2jBF5LFW7U67dhp45n'}</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTSQTuDmtmTQNDwTJX'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2jAd7iVbsTydkohj5B'}</t>
         </is>
       </c>
     </row>
@@ -15139,7 +15139,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTTkpZbcJRe2MZQiu4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2jBwjxSAPBFNd1xcJi'}</t>
         </is>
       </c>
     </row>
@@ -15186,7 +15186,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzTUiNX9eM6bZ64ZkNt'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2jCeuWcEsxrPGcvT55'}</t>
         </is>
       </c>
     </row>
@@ -15233,7 +15233,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPYxkKBBvgDf1vFKyX'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2epCvrUvFfWbMxZFtH'}</t>
         </is>
       </c>
     </row>
@@ -15280,7 +15280,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzPZdBWVyYAeBEwinuH'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2epmuRdG1GqGaS7LqL'}</t>
         </is>
       </c>
     </row>
@@ -15327,7 +15327,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzSgdCmeSUhDdC7Jcbg'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i82KfDUgc5V163ABi'}</t>
         </is>
       </c>
     </row>
@@ -15374,7 +15374,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzShDv5STk6UZNWNYdv'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i8bo2hFgQAnXhpThG'}</t>
         </is>
       </c>
     </row>
@@ -15421,7 +15421,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfzShmAFUTdWbFkaGHA4'}</t>
+          <t>Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011Cbg2i9C22qewpy4C3JHaZ'}</t>
         </is>
       </c>
     </row>
@@ -16403,7 +16403,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>03/06/2026 08:13</t>
+          <t>03/06/2026 08:43</t>
         </is>
       </c>
     </row>

</xml_diff>